<commit_message>
fix template / example mixup
</commit_message>
<xml_diff>
--- a/data/Restoration_Monitoring_Cover_EXAMPLE.xlsx
+++ b/data/Restoration_Monitoring_Cover_EXAMPLE.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://doimspp.sharepoint.com/sites/usgs-carbonate_budget_restoration_tool/Shared Documents/Carbonate Budget Tool Collaboration/Carbonate_Budget_Tool_Code/CarbonateBudgetRestorationTool/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\__git\CBuRT\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="28" documentId="8_{31D97D8A-81BF-4130-9925-67CFAF7DC92E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5DBA3E52-CC7C-441C-A16F-45E19E2260C7}"/>
+  <xr:revisionPtr revIDLastSave="95" documentId="8_{31D97D8A-81BF-4130-9925-67CFAF7DC92E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1131F112-0661-40A2-9965-DFCB4BEF0F46}"/>
   <bookViews>
-    <workbookView xWindow="14317" yWindow="0" windowWidth="14565" windowHeight="17363" activeTab="1" xr2:uid="{0278FB9D-D97A-43A8-AA68-A0B70EFAF30B}"/>
+    <workbookView xWindow="57480" yWindow="22020" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{0278FB9D-D97A-43A8-AA68-A0B70EFAF30B}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="3" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="122">
   <si>
     <t>Acropora cervicornis</t>
   </si>
@@ -1218,6 +1218,766 @@
         <v>1.3480392160000001</v>
       </c>
     </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>118</v>
+      </c>
+      <c r="B7" t="s">
+        <v>119</v>
+      </c>
+      <c r="C7" s="6">
+        <v>24.459129999999998</v>
+      </c>
+      <c r="D7" s="6">
+        <v>-81.845830000000007</v>
+      </c>
+      <c r="E7" t="s">
+        <v>106</v>
+      </c>
+      <c r="F7" t="s">
+        <v>113</v>
+      </c>
+      <c r="G7">
+        <v>100</v>
+      </c>
+      <c r="H7" t="s">
+        <v>120</v>
+      </c>
+      <c r="I7" t="s">
+        <v>121</v>
+      </c>
+      <c r="J7">
+        <v>1</v>
+      </c>
+      <c r="K7" t="s">
+        <v>0</v>
+      </c>
+      <c r="L7">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>118</v>
+      </c>
+      <c r="B8" t="s">
+        <v>119</v>
+      </c>
+      <c r="C8" s="6">
+        <v>24.459129999999998</v>
+      </c>
+      <c r="D8" s="6">
+        <v>-81.845830000000007</v>
+      </c>
+      <c r="E8" t="s">
+        <v>106</v>
+      </c>
+      <c r="F8" t="s">
+        <v>113</v>
+      </c>
+      <c r="G8">
+        <v>100</v>
+      </c>
+      <c r="H8" t="s">
+        <v>120</v>
+      </c>
+      <c r="I8" t="s">
+        <v>121</v>
+      </c>
+      <c r="J8">
+        <v>3</v>
+      </c>
+      <c r="K8" t="s">
+        <v>1</v>
+      </c>
+      <c r="L8">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>118</v>
+      </c>
+      <c r="B9" t="s">
+        <v>119</v>
+      </c>
+      <c r="C9" s="6">
+        <v>24.459129999999998</v>
+      </c>
+      <c r="D9" s="6">
+        <v>-81.845830000000007</v>
+      </c>
+      <c r="E9" t="s">
+        <v>106</v>
+      </c>
+      <c r="F9" t="s">
+        <v>113</v>
+      </c>
+      <c r="G9">
+        <v>100</v>
+      </c>
+      <c r="H9" t="s">
+        <v>120</v>
+      </c>
+      <c r="I9" t="s">
+        <v>121</v>
+      </c>
+      <c r="J9">
+        <v>3</v>
+      </c>
+      <c r="K9" t="s">
+        <v>0</v>
+      </c>
+      <c r="L9">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
+        <v>118</v>
+      </c>
+      <c r="B10" t="s">
+        <v>119</v>
+      </c>
+      <c r="C10" s="6">
+        <v>24.459129999999998</v>
+      </c>
+      <c r="D10" s="6">
+        <v>-81.845830000000007</v>
+      </c>
+      <c r="E10" t="s">
+        <v>106</v>
+      </c>
+      <c r="F10" t="s">
+        <v>113</v>
+      </c>
+      <c r="G10">
+        <v>100</v>
+      </c>
+      <c r="H10" t="s">
+        <v>120</v>
+      </c>
+      <c r="I10" t="s">
+        <v>121</v>
+      </c>
+      <c r="J10">
+        <v>3</v>
+      </c>
+      <c r="K10" t="s">
+        <v>44</v>
+      </c>
+      <c r="L10">
+        <v>2.95</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
+        <v>118</v>
+      </c>
+      <c r="B11" t="s">
+        <v>119</v>
+      </c>
+      <c r="C11" s="6">
+        <v>24.459129999999998</v>
+      </c>
+      <c r="D11" s="6">
+        <v>-81.845830000000007</v>
+      </c>
+      <c r="E11" t="s">
+        <v>106</v>
+      </c>
+      <c r="F11" t="s">
+        <v>113</v>
+      </c>
+      <c r="G11">
+        <v>100</v>
+      </c>
+      <c r="H11" t="s">
+        <v>120</v>
+      </c>
+      <c r="I11" t="s">
+        <v>121</v>
+      </c>
+      <c r="J11">
+        <v>3</v>
+      </c>
+      <c r="K11" t="s">
+        <v>42</v>
+      </c>
+      <c r="L11">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A12" t="s">
+        <v>118</v>
+      </c>
+      <c r="B12" t="s">
+        <v>119</v>
+      </c>
+      <c r="C12" s="6">
+        <v>24.459129999999998</v>
+      </c>
+      <c r="D12" s="6">
+        <v>-81.845830000000007</v>
+      </c>
+      <c r="E12" t="s">
+        <v>106</v>
+      </c>
+      <c r="F12" t="s">
+        <v>113</v>
+      </c>
+      <c r="G12">
+        <v>100</v>
+      </c>
+      <c r="H12" t="s">
+        <v>120</v>
+      </c>
+      <c r="I12" t="s">
+        <v>121</v>
+      </c>
+      <c r="J12">
+        <v>5</v>
+      </c>
+      <c r="K12" t="s">
+        <v>1</v>
+      </c>
+      <c r="L12">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A13" t="s">
+        <v>118</v>
+      </c>
+      <c r="B13" t="s">
+        <v>119</v>
+      </c>
+      <c r="C13" s="6">
+        <v>24.459129999999998</v>
+      </c>
+      <c r="D13" s="6">
+        <v>-81.845830000000007</v>
+      </c>
+      <c r="E13" t="s">
+        <v>106</v>
+      </c>
+      <c r="F13" t="s">
+        <v>113</v>
+      </c>
+      <c r="G13">
+        <v>100</v>
+      </c>
+      <c r="H13" t="s">
+        <v>120</v>
+      </c>
+      <c r="I13" t="s">
+        <v>121</v>
+      </c>
+      <c r="J13">
+        <v>5</v>
+      </c>
+      <c r="K13" t="s">
+        <v>0</v>
+      </c>
+      <c r="L13">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A14" t="s">
+        <v>118</v>
+      </c>
+      <c r="B14" t="s">
+        <v>119</v>
+      </c>
+      <c r="C14" s="6">
+        <v>24.459129999999998</v>
+      </c>
+      <c r="D14" s="6">
+        <v>-81.845830000000007</v>
+      </c>
+      <c r="E14" t="s">
+        <v>106</v>
+      </c>
+      <c r="F14" t="s">
+        <v>113</v>
+      </c>
+      <c r="G14">
+        <v>100</v>
+      </c>
+      <c r="H14" t="s">
+        <v>120</v>
+      </c>
+      <c r="I14" t="s">
+        <v>121</v>
+      </c>
+      <c r="J14">
+        <v>5</v>
+      </c>
+      <c r="K14" t="s">
+        <v>44</v>
+      </c>
+      <c r="L14">
+        <v>2.8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A15" t="s">
+        <v>118</v>
+      </c>
+      <c r="B15" t="s">
+        <v>119</v>
+      </c>
+      <c r="C15" s="6">
+        <v>24.459129999999998</v>
+      </c>
+      <c r="D15" s="6">
+        <v>-81.845830000000007</v>
+      </c>
+      <c r="E15" t="s">
+        <v>106</v>
+      </c>
+      <c r="F15" t="s">
+        <v>113</v>
+      </c>
+      <c r="G15">
+        <v>100</v>
+      </c>
+      <c r="H15" t="s">
+        <v>120</v>
+      </c>
+      <c r="I15" t="s">
+        <v>121</v>
+      </c>
+      <c r="J15">
+        <v>5</v>
+      </c>
+      <c r="K15" t="s">
+        <v>42</v>
+      </c>
+      <c r="L15">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A16" t="s">
+        <v>118</v>
+      </c>
+      <c r="B16" t="s">
+        <v>119</v>
+      </c>
+      <c r="C16" s="6">
+        <v>24.459129999999998</v>
+      </c>
+      <c r="D16" s="6">
+        <v>-81.845830000000007</v>
+      </c>
+      <c r="E16" t="s">
+        <v>106</v>
+      </c>
+      <c r="F16" t="s">
+        <v>113</v>
+      </c>
+      <c r="G16">
+        <v>100</v>
+      </c>
+      <c r="H16" t="s">
+        <v>120</v>
+      </c>
+      <c r="I16" t="s">
+        <v>121</v>
+      </c>
+      <c r="J16">
+        <v>5</v>
+      </c>
+      <c r="K16" t="s">
+        <v>55</v>
+      </c>
+      <c r="L16">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A17" t="s">
+        <v>118</v>
+      </c>
+      <c r="B17" t="s">
+        <v>119</v>
+      </c>
+      <c r="C17" s="6">
+        <v>24.459129999999998</v>
+      </c>
+      <c r="D17" s="6">
+        <v>-81.845830000000007</v>
+      </c>
+      <c r="E17" t="s">
+        <v>106</v>
+      </c>
+      <c r="F17" t="s">
+        <v>113</v>
+      </c>
+      <c r="G17">
+        <v>100</v>
+      </c>
+      <c r="H17" t="s">
+        <v>120</v>
+      </c>
+      <c r="I17" t="s">
+        <v>121</v>
+      </c>
+      <c r="J17">
+        <v>10</v>
+      </c>
+      <c r="K17" t="s">
+        <v>1</v>
+      </c>
+      <c r="L17">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A18" t="s">
+        <v>118</v>
+      </c>
+      <c r="B18" t="s">
+        <v>119</v>
+      </c>
+      <c r="C18" s="6">
+        <v>24.459129999999998</v>
+      </c>
+      <c r="D18" s="6">
+        <v>-81.845830000000007</v>
+      </c>
+      <c r="E18" t="s">
+        <v>106</v>
+      </c>
+      <c r="F18" t="s">
+        <v>113</v>
+      </c>
+      <c r="G18">
+        <v>100</v>
+      </c>
+      <c r="H18" t="s">
+        <v>120</v>
+      </c>
+      <c r="I18" t="s">
+        <v>121</v>
+      </c>
+      <c r="J18">
+        <v>10</v>
+      </c>
+      <c r="K18" t="s">
+        <v>0</v>
+      </c>
+      <c r="L18">
+        <v>1.75</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A19" t="s">
+        <v>118</v>
+      </c>
+      <c r="B19" t="s">
+        <v>119</v>
+      </c>
+      <c r="C19" s="6">
+        <v>24.459129999999998</v>
+      </c>
+      <c r="D19" s="6">
+        <v>-81.845830000000007</v>
+      </c>
+      <c r="E19" t="s">
+        <v>106</v>
+      </c>
+      <c r="F19" t="s">
+        <v>113</v>
+      </c>
+      <c r="G19">
+        <v>100</v>
+      </c>
+      <c r="H19" t="s">
+        <v>120</v>
+      </c>
+      <c r="I19" t="s">
+        <v>121</v>
+      </c>
+      <c r="J19">
+        <v>10</v>
+      </c>
+      <c r="K19" t="s">
+        <v>44</v>
+      </c>
+      <c r="L19">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A20" t="s">
+        <v>118</v>
+      </c>
+      <c r="B20" t="s">
+        <v>119</v>
+      </c>
+      <c r="C20" s="6">
+        <v>24.459129999999998</v>
+      </c>
+      <c r="D20" s="6">
+        <v>-81.845830000000007</v>
+      </c>
+      <c r="E20" t="s">
+        <v>106</v>
+      </c>
+      <c r="F20" t="s">
+        <v>113</v>
+      </c>
+      <c r="G20">
+        <v>100</v>
+      </c>
+      <c r="H20" t="s">
+        <v>120</v>
+      </c>
+      <c r="I20" t="s">
+        <v>121</v>
+      </c>
+      <c r="J20">
+        <v>10</v>
+      </c>
+      <c r="K20" t="s">
+        <v>42</v>
+      </c>
+      <c r="L20">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A21" t="s">
+        <v>118</v>
+      </c>
+      <c r="B21" t="s">
+        <v>119</v>
+      </c>
+      <c r="C21" s="6">
+        <v>24.459129999999998</v>
+      </c>
+      <c r="D21" s="6">
+        <v>-81.845830000000007</v>
+      </c>
+      <c r="E21" t="s">
+        <v>106</v>
+      </c>
+      <c r="F21" t="s">
+        <v>113</v>
+      </c>
+      <c r="G21">
+        <v>100</v>
+      </c>
+      <c r="H21" t="s">
+        <v>120</v>
+      </c>
+      <c r="I21" t="s">
+        <v>121</v>
+      </c>
+      <c r="J21">
+        <v>10</v>
+      </c>
+      <c r="K21" t="s">
+        <v>55</v>
+      </c>
+      <c r="L21">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A22" t="s">
+        <v>118</v>
+      </c>
+      <c r="B22" t="s">
+        <v>119</v>
+      </c>
+      <c r="C22" s="6">
+        <v>24.459129999999998</v>
+      </c>
+      <c r="D22" s="6">
+        <v>-81.845830000000007</v>
+      </c>
+      <c r="E22" t="s">
+        <v>106</v>
+      </c>
+      <c r="F22" t="s">
+        <v>113</v>
+      </c>
+      <c r="G22">
+        <v>100</v>
+      </c>
+      <c r="H22" t="s">
+        <v>120</v>
+      </c>
+      <c r="I22" t="s">
+        <v>121</v>
+      </c>
+      <c r="J22">
+        <v>-1</v>
+      </c>
+      <c r="K22" t="s">
+        <v>85</v>
+      </c>
+      <c r="L22">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A23" t="s">
+        <v>118</v>
+      </c>
+      <c r="B23" t="s">
+        <v>119</v>
+      </c>
+      <c r="C23" s="6">
+        <v>24.459129999999998</v>
+      </c>
+      <c r="D23" s="6">
+        <v>-81.845830000000007</v>
+      </c>
+      <c r="E23" t="s">
+        <v>106</v>
+      </c>
+      <c r="F23" t="s">
+        <v>113</v>
+      </c>
+      <c r="G23">
+        <v>100</v>
+      </c>
+      <c r="H23" t="s">
+        <v>120</v>
+      </c>
+      <c r="I23" t="s">
+        <v>121</v>
+      </c>
+      <c r="J23">
+        <v>1</v>
+      </c>
+      <c r="K23" t="s">
+        <v>85</v>
+      </c>
+      <c r="L23">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A24" t="s">
+        <v>118</v>
+      </c>
+      <c r="B24" t="s">
+        <v>119</v>
+      </c>
+      <c r="C24" s="6">
+        <v>24.459129999999998</v>
+      </c>
+      <c r="D24" s="6">
+        <v>-81.845830000000007</v>
+      </c>
+      <c r="E24" t="s">
+        <v>106</v>
+      </c>
+      <c r="F24" t="s">
+        <v>113</v>
+      </c>
+      <c r="G24">
+        <v>100</v>
+      </c>
+      <c r="H24" t="s">
+        <v>120</v>
+      </c>
+      <c r="I24" t="s">
+        <v>121</v>
+      </c>
+      <c r="J24">
+        <v>3</v>
+      </c>
+      <c r="K24" t="s">
+        <v>85</v>
+      </c>
+      <c r="L24">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A25" t="s">
+        <v>118</v>
+      </c>
+      <c r="B25" t="s">
+        <v>119</v>
+      </c>
+      <c r="C25" s="6">
+        <v>24.459129999999998</v>
+      </c>
+      <c r="D25" s="6">
+        <v>-81.845830000000007</v>
+      </c>
+      <c r="E25" t="s">
+        <v>106</v>
+      </c>
+      <c r="F25" t="s">
+        <v>113</v>
+      </c>
+      <c r="G25">
+        <v>100</v>
+      </c>
+      <c r="H25" t="s">
+        <v>120</v>
+      </c>
+      <c r="I25" t="s">
+        <v>121</v>
+      </c>
+      <c r="J25">
+        <v>5</v>
+      </c>
+      <c r="K25" t="s">
+        <v>85</v>
+      </c>
+      <c r="L25">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A26" t="s">
+        <v>118</v>
+      </c>
+      <c r="B26" t="s">
+        <v>119</v>
+      </c>
+      <c r="C26" s="6">
+        <v>24.459129999999998</v>
+      </c>
+      <c r="D26" s="6">
+        <v>-81.845830000000007</v>
+      </c>
+      <c r="E26" t="s">
+        <v>106</v>
+      </c>
+      <c r="F26" t="s">
+        <v>113</v>
+      </c>
+      <c r="G26">
+        <v>100</v>
+      </c>
+      <c r="H26" t="s">
+        <v>120</v>
+      </c>
+      <c r="I26" t="s">
+        <v>121</v>
+      </c>
+      <c r="J26">
+        <v>10</v>
+      </c>
+      <c r="K26" t="s">
+        <v>85</v>
+      </c>
+      <c r="L26">
+        <v>0.5</v>
+      </c>
+    </row>
     <row r="40" spans="21:21" x14ac:dyDescent="0.45">
       <c r="U40" s="2"/>
     </row>
@@ -1230,7 +1990,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F1048576" xr:uid="{B3D722F7-1AC4-4F85-A533-096480B6E937}">
       <formula1>"Inshore, MidChannel, Offshore, Bank, Lagoon, ForeReef"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E6" xr:uid="{FC4BDEA1-B79E-4B46-931A-F54681159ED2}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E26" xr:uid="{FC4BDEA1-B79E-4B46-931A-F54681159ED2}">
       <formula1>"DryTortugas, LowerKeys,MiddleKeys, UpperKeys, Biscayne, SoutheastFlorida"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1248,7 +2008,7 @@
           <x14:formula1>
             <xm:f>Metadata!A2:A7</xm:f>
           </x14:formula1>
-          <xm:sqref>E1 E7:E1048576</xm:sqref>
+          <xm:sqref>E1 E27:E1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1734,8 +2494,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000AA90A7536739341825FB392424435FB" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ca57789ecb406bb7a99068f68ac4c0ed">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="797e7fd4-719a-42b3-b312-968ffa9058ad" xmlns:ns3="811eef35-9bdd-441e-81aa-50455f68c6c3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="89dc4794f4784a0bac47690674a3da53" ns2:_="" ns3:_="">
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000AA90A7536739341825FB392424435FB" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="647735499ae6baa62e6fc7f5ed3567b4">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="797e7fd4-719a-42b3-b312-968ffa9058ad" xmlns:ns3="811eef35-9bdd-441e-81aa-50455f68c6c3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="47ff4a2bf1fedf465812d90a21a07c12" ns2:_="" ns3:_="">
     <xsd:import namespace="797e7fd4-719a-42b3-b312-968ffa9058ad"/>
     <xsd:import namespace="811eef35-9bdd-441e-81aa-50455f68c6c3"/>
     <xsd:element name="properties">
@@ -1928,15 +2697,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1949,7 +2709,15 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7D5B4E66-2F53-40AB-B6DF-59838CE46951}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5D6BB395-747F-41BC-A23A-168993E4FE92}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4ABA30CC-C1F2-488C-BE05-7ED5EA282AA6}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
@@ -1963,14 +2731,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5D6BB395-747F-41BC-A23A-168993E4FE92}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>